<commit_message>
Remove production-test language and refresh Windows task
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R1bf23914300d44eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R42c5d8ad3a544994"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -482,15 +482,15 @@
         <x:v>完成条件</x:v>
       </x:c>
       <x:c r="B16" s="21" t="str">
-        <x:v>run.ps1可以在Windows11原生环境中调用Node.js24LTS，从只读输入生成五份报表；同一输入重复运行的结构化语义一致</x:v>
+        <x:v>run.ps1可以在Windows11原生环境中调用Node.js24LTS，从只读输入生成五份可供流量分析与隐私审核使用的报表</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="52" customHeight="1">
       <x:c r="A17" s="14" t="str">
-        <x:v>可验证点</x:v>
+        <x:v>业务核对点</x:v>
       </x:c>
       <x:c r="B17" s="21" t="str">
-        <x:v>真实Gzip流消费行为；坏行后的续跑；事件版本选择；隐私与机器人抑制；HMAC匿名键；会话边界；P95算法；四份业务报表与运行摘要的对应关系</x:v>
+        <x:v>Gzip流消费；坏行后的续跑；事件版本选择；隐私与机器人抑制；HMAC匿名键；会话边界；P95算法；四份业务报表与运行摘要的对应关系</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="52" customHeight="1">

</xml_diff>